<commit_message>
fix: correct expense tracker data to match actual logs
- All Credit Card → Debit Card
- Reviews confirmed Venmo
- Fixed dates to match Google Sheet exactly
- Removed duplicate entries I invented (2nd Pearson, 2nd Insurance, etc.)
- Added missing Quo $1 entry (1/14/26)
- Corrected gas amounts to actual values ($22.68, $25.82, etc.)
- 26 expense entries + 8 gas entries now match source of truth

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TotalGuard_2026_Expense_Tracker.xlsx
+++ b/TotalGuard_2026_Expense_Tracker.xlsx
@@ -735,7 +735,7 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Quo phone app</t>
+          <t>Quo (phone app)</t>
         </is>
       </c>
       <c r="E3" s="6" t="n">
@@ -743,7 +743,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>ACH/Bank</t>
+          <t>Debit Card</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
@@ -777,20 +777,20 @@
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Software/SaaS</t>
+          <t>Phone/Communications</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>Lovable Website Builder</t>
+          <t>Quo (phone app)</t>
         </is>
       </c>
       <c r="E4" s="10" t="n">
-        <v>15</v>
+        <v>19.5</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>Debit Card</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="I4" s="9" t="inlineStr">
         <is>
-          <t>Line 27a - Other Expenses</t>
+          <t>Line 25 - Utilities</t>
         </is>
       </c>
       <c r="J4" s="9" t="inlineStr">
@@ -820,29 +820,29 @@
         <v>3</v>
       </c>
       <c r="B5" s="4" t="n">
-        <v>46032</v>
+        <v>46036</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Software/SaaS</t>
+          <t>Phone/Communications</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Porkbun Domains</t>
+          <t>Quo</t>
         </is>
       </c>
       <c r="E5" s="6" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>Debit Card</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Annual</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Line 27a - Other Expenses</t>
+          <t>Line 25 - Utilities</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
@@ -867,29 +867,29 @@
         <v>4</v>
       </c>
       <c r="B6" s="8" t="n">
-        <v>46037</v>
+        <v>46051</v>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Training/Education</t>
+          <t>Software/SaaS</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Pearson VUE exam</t>
+          <t>Lovable Website Builder</t>
         </is>
       </c>
       <c r="E6" s="10" t="n">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>Debit Card</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>One-Time</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="H6" s="9" t="inlineStr">
@@ -914,29 +914,29 @@
         <v>5</v>
       </c>
       <c r="B7" s="4" t="n">
-        <v>46037</v>
+        <v>46052</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Licensing/Permits</t>
+          <t>Software/SaaS</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>License application fee</t>
+          <t>Chat subscription</t>
         </is>
       </c>
       <c r="E7" s="6" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>Debit Card</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>One-Time</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -961,29 +961,29 @@
         <v>6</v>
       </c>
       <c r="B8" s="8" t="n">
-        <v>46042</v>
+        <v>46053</v>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Insurance</t>
+          <t>Software/SaaS</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>Pekin Liability Insurance</t>
+          <t>Lovable Website Builder</t>
         </is>
       </c>
       <c r="E8" s="10" t="n">
-        <v>86</v>
+        <v>12.5</v>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>ACH/Bank</t>
+          <t>Debit Card</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>Annual</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="H8" s="9" t="inlineStr">
@@ -993,7 +993,7 @@
       </c>
       <c r="I8" s="9" t="inlineStr">
         <is>
-          <t>Line 15 - Insurance</t>
+          <t>Line 27a - Other Expenses</t>
         </is>
       </c>
       <c r="J8" s="9" t="inlineStr">
@@ -1008,7 +1008,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="4" t="n">
-        <v>46042</v>
+        <v>46057</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
@@ -1017,15 +1017,15 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Lovable Website Builder</t>
+          <t>Brevo (marketing)</t>
         </is>
       </c>
       <c r="E9" s="6" t="n">
-        <v>12.5</v>
+        <v>9</v>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>Debit Card</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -1040,7 +1040,7 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Line 27a - Other Expenses</t>
+          <t>Line 8 - Advertising</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
@@ -1055,24 +1055,24 @@
         <v>8</v>
       </c>
       <c r="B10" s="8" t="n">
-        <v>46047</v>
+        <v>46059</v>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Marketing/Advertising</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Reviews ($5/per)</t>
         </is>
       </c>
       <c r="E10" s="10" t="n">
-        <v>105</v>
+        <v>45</v>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>Venmo</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="I10" s="9" t="inlineStr">
         <is>
-          <t>Line 22 - Supplies</t>
+          <t>Line 8 - Advertising</t>
         </is>
       </c>
       <c r="J10" s="9" t="inlineStr">
@@ -1102,24 +1102,24 @@
         <v>9</v>
       </c>
       <c r="B11" s="4" t="n">
-        <v>46052</v>
+        <v>46062</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Software/SaaS</t>
+          <t>Phone/Communications</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Chat subscription</t>
+          <t>Quo (Biz phone)</t>
         </is>
       </c>
       <c r="E11" s="6" t="n">
-        <v>20</v>
+        <v>22.01</v>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>ACH/Bank</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
@@ -1134,7 +1134,7 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Line 27a - Other Expenses</t>
+          <t>Line 25 - Utilities</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
@@ -1149,24 +1149,24 @@
         <v>10</v>
       </c>
       <c r="B12" s="8" t="n">
-        <v>46054</v>
+        <v>46062</v>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Software/SaaS</t>
+          <t>Phone/Communications</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>Claude Code</t>
+          <t>Quo</t>
         </is>
       </c>
       <c r="E12" s="10" t="n">
-        <v>100</v>
+        <v>22.01</v>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>ACH/Bank</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
@@ -1181,7 +1181,7 @@
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>Line 27a - Other Expenses</t>
+          <t>Line 25 - Utilities</t>
         </is>
       </c>
       <c r="J12" s="9" t="inlineStr">
@@ -1196,7 +1196,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="4" t="n">
-        <v>46054</v>
+        <v>46065</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
@@ -1205,15 +1205,15 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Brevo marketing</t>
+          <t>Lovable Website Builder</t>
         </is>
       </c>
       <c r="E13" s="6" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>Debit Card</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Line 8 - Advertising</t>
+          <t>Line 27a - Other Expenses</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
@@ -1243,7 +1243,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="8" t="n">
-        <v>46054</v>
+        <v>46076</v>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
@@ -1252,15 +1252,15 @@
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>n8n</t>
+          <t>Claude Code</t>
         </is>
       </c>
       <c r="E14" s="10" t="n">
-        <v>24</v>
+        <v>100</v>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>Debit Card</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
@@ -1290,29 +1290,29 @@
         <v>13</v>
       </c>
       <c r="B15" s="4" t="n">
-        <v>46054</v>
+        <v>46077</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Phone/Communications</t>
+          <t>Training/Education</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Twilio</t>
+          <t>Pearson VUE exam</t>
         </is>
       </c>
       <c r="E15" s="6" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>Debit Card</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>One-Time</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>Line 25 - Utilities</t>
+          <t>Line 27a - Other Expenses</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
@@ -1337,29 +1337,29 @@
         <v>14</v>
       </c>
       <c r="B16" s="8" t="n">
-        <v>46054</v>
+        <v>46081</v>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Marketing/Advertising</t>
+          <t>Software/SaaS</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Reviews ($5/per)</t>
+          <t>Lovable Website Builder</t>
         </is>
       </c>
       <c r="E16" s="10" t="n">
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>Venmo</t>
+          <t>Debit Card</t>
         </is>
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t>One-Time</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="H16" s="9" t="inlineStr">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="I16" s="9" t="inlineStr">
         <is>
-          <t>Line 8 - Advertising</t>
+          <t>Line 27a - Other Expenses</t>
         </is>
       </c>
       <c r="J16" s="9" t="inlineStr">
@@ -1384,29 +1384,29 @@
         <v>15</v>
       </c>
       <c r="B17" s="4" t="n">
-        <v>46054</v>
+        <v>46081</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Software/SaaS</t>
+          <t>Equipment</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Lovable Website Builder</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="E17" s="6" t="n">
-        <v>30</v>
+        <v>105</v>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>Debit Card</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>One-Time</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>Line 27a - Other Expenses</t>
+          <t>Line 22 - Supplies</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
@@ -1431,24 +1431,24 @@
         <v>16</v>
       </c>
       <c r="B18" s="8" t="n">
-        <v>46062</v>
+        <v>46086</v>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Phone/Communications</t>
+          <t>Software/SaaS</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Quo (Biz phone)</t>
+          <t>Jobber Subscription</t>
         </is>
       </c>
       <c r="E18" s="10" t="n">
-        <v>22.01</v>
+        <v>49</v>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>ACH/Bank</t>
+          <t>Debit Card</t>
         </is>
       </c>
       <c r="G18" s="9" t="inlineStr">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="I18" s="9" t="inlineStr">
         <is>
-          <t>Line 25 - Utilities</t>
+          <t>Line 27a - Other Expenses</t>
         </is>
       </c>
       <c r="J18" s="9" t="inlineStr">
@@ -1478,29 +1478,29 @@
         <v>17</v>
       </c>
       <c r="B19" s="4" t="n">
-        <v>46065</v>
+        <v>46086</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Software/SaaS</t>
+          <t>Licensing/Permits</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Lovable Website Builder</t>
+          <t>Licence application fee</t>
         </is>
       </c>
       <c r="E19" s="6" t="n">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>Debit Card</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>One-Time</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
@@ -1525,29 +1525,29 @@
         <v>18</v>
       </c>
       <c r="B20" s="8" t="n">
-        <v>46073</v>
+        <v>46088</v>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Insurance</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>Trailer 5x10</t>
+          <t>Pekin Liability Insurance</t>
         </is>
       </c>
       <c r="E20" s="10" t="n">
-        <v>1582</v>
+        <v>86</v>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>ACH/Bank</t>
         </is>
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>One-Time</t>
+          <t>Annual</t>
         </is>
       </c>
       <c r="H20" s="9" t="inlineStr">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="I20" s="9" t="inlineStr">
         <is>
-          <t>Line 22 - Supplies</t>
+          <t>Line 15 - Insurance</t>
         </is>
       </c>
       <c r="J20" s="9" t="inlineStr">
@@ -1572,7 +1572,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="4" t="n">
-        <v>46076</v>
+        <v>46088</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
@@ -1581,20 +1581,20 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Claude Code</t>
+          <t>Porkbun Domains</t>
         </is>
       </c>
       <c r="E21" s="6" t="n">
-        <v>100</v>
+        <v>22</v>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>Debit Card</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Annual</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
@@ -1619,24 +1619,24 @@
         <v>20</v>
       </c>
       <c r="B22" s="8" t="n">
-        <v>46077</v>
+        <v>46089</v>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Training/Education</t>
+          <t>Marketing/Advertising</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Pearson VUE exam</t>
+          <t>1x G Review</t>
         </is>
       </c>
       <c r="E22" s="10" t="n">
-        <v>45</v>
+        <v>5</v>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>Venmo</t>
         </is>
       </c>
       <c r="G22" s="9" t="inlineStr">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>Line 27a - Other Expenses</t>
+          <t>Line 8 - Advertising</t>
         </is>
       </c>
       <c r="J22" s="9" t="inlineStr">
@@ -1666,29 +1666,29 @@
         <v>21</v>
       </c>
       <c r="B23" s="4" t="n">
-        <v>46078</v>
+        <v>46090</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Phone/Communications</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Trailer Hooks</t>
+          <t>Twilio</t>
         </is>
       </c>
       <c r="E23" s="6" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>Debit Card</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>One-Time</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>Line 22 - Supplies</t>
+          <t>Line 25 - Utilities</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr">
@@ -1713,24 +1713,24 @@
         <v>22</v>
       </c>
       <c r="B24" s="8" t="n">
-        <v>46081</v>
+        <v>46090</v>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Software/SaaS</t>
+          <t>Phone/Communications</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Lovable Website Builder</t>
+          <t>Quo</t>
         </is>
       </c>
       <c r="E24" s="10" t="n">
-        <v>13</v>
+        <v>22.01</v>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>ACH/Bank</t>
         </is>
       </c>
       <c r="G24" s="9" t="inlineStr">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="I24" s="9" t="inlineStr">
         <is>
-          <t>Line 27a - Other Expenses</t>
+          <t>Line 25 - Utilities</t>
         </is>
       </c>
       <c r="J24" s="9" t="inlineStr">
@@ -1760,24 +1760,24 @@
         <v>23</v>
       </c>
       <c r="B25" s="4" t="n">
-        <v>46081</v>
+        <v>46091</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Marketing/Advertising</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Monitor (2nd)</t>
+          <t>Yard Signs Uz Marketing</t>
         </is>
       </c>
       <c r="E25" s="6" t="n">
-        <v>105</v>
+        <v>398</v>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>Check</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -1792,7 +1792,7 @@
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>Line 22 - Supplies</t>
+          <t>Line 8 - Advertising</t>
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr">
@@ -1807,20 +1807,20 @@
         <v>24</v>
       </c>
       <c r="B26" s="8" t="n">
-        <v>46082</v>
+        <v>46092</v>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Marketing/Advertising</t>
+          <t>Equipment</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>Yard Signs Uz Marketing</t>
+          <t>Trailer 5 x 10 (dad)</t>
         </is>
       </c>
       <c r="E26" s="10" t="n">
-        <v>398</v>
+        <v>1582</v>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
@@ -1839,7 +1839,7 @@
       </c>
       <c r="I26" s="9" t="inlineStr">
         <is>
-          <t>Line 8 - Advertising</t>
+          <t>Line 22 - Supplies</t>
         </is>
       </c>
       <c r="J26" s="9" t="inlineStr">
@@ -1854,29 +1854,29 @@
         <v>25</v>
       </c>
       <c r="B27" s="4" t="n">
-        <v>46082</v>
+        <v>46092</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Software/SaaS</t>
+          <t>Equipment</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Jobber Subscription</t>
+          <t>Trailer Hooks</t>
         </is>
       </c>
       <c r="E27" s="6" t="n">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>One-Time</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>Line 27a - Other Expenses</t>
+          <t>Line 22 - Supplies</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr">
@@ -1901,29 +1901,29 @@
         <v>26</v>
       </c>
       <c r="B28" s="8" t="n">
-        <v>46086</v>
+        <v>46092</v>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Licensing/Permits</t>
+          <t>Software/SaaS</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>License application fee</t>
+          <t>n8n</t>
         </is>
       </c>
       <c r="E28" s="10" t="n">
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>Debit Card</t>
         </is>
       </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t>One-Time</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="H28" s="9" t="inlineStr">
@@ -1947,282 +1947,90 @@
       <c r="A29" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="B29" s="4" t="n">
-        <v>46087</v>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>Marketing/Advertising</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>Reviews ($5/per)</t>
-        </is>
-      </c>
-      <c r="E29" s="6" t="n">
-        <v>45</v>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="G29" s="5" t="inlineStr">
-        <is>
-          <t>One-Time</t>
-        </is>
-      </c>
-      <c r="H29" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I29" s="5" t="inlineStr">
-        <is>
-          <t>Line 8 - Advertising</t>
-        </is>
-      </c>
-      <c r="J29" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="B29" s="4" t="n"/>
+      <c r="C29" s="5" t="n"/>
+      <c r="D29" s="5" t="n"/>
+      <c r="E29" s="6" t="n"/>
+      <c r="F29" s="5" t="n"/>
+      <c r="G29" s="5" t="n"/>
+      <c r="H29" s="5" t="n"/>
+      <c r="I29" s="5" t="n"/>
+      <c r="J29" s="5" t="n"/>
       <c r="K29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n">
         <v>28</v>
       </c>
-      <c r="B30" s="8" t="n">
-        <v>46088</v>
-      </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>Insurance</t>
-        </is>
-      </c>
-      <c r="D30" s="9" t="inlineStr">
-        <is>
-          <t>Pekin Liability Insurance</t>
-        </is>
-      </c>
-      <c r="E30" s="10" t="n">
-        <v>86</v>
-      </c>
-      <c r="F30" s="9" t="inlineStr">
-        <is>
-          <t>ACH/Bank</t>
-        </is>
-      </c>
-      <c r="G30" s="9" t="inlineStr">
-        <is>
-          <t>Annual</t>
-        </is>
-      </c>
-      <c r="H30" s="9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I30" s="9" t="inlineStr">
-        <is>
-          <t>Line 15 - Insurance</t>
-        </is>
-      </c>
-      <c r="J30" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="B30" s="8" t="n"/>
+      <c r="C30" s="9" t="n"/>
+      <c r="D30" s="9" t="n"/>
+      <c r="E30" s="10" t="n"/>
+      <c r="F30" s="9" t="n"/>
+      <c r="G30" s="9" t="n"/>
+      <c r="H30" s="9" t="n"/>
+      <c r="I30" s="9" t="n"/>
+      <c r="J30" s="9" t="n"/>
       <c r="K30" s="9" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="B31" s="4" t="n">
-        <v>46088</v>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>Software/SaaS</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>Porkbun Domains</t>
-        </is>
-      </c>
-      <c r="E31" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>Credit Card</t>
-        </is>
-      </c>
-      <c r="G31" s="5" t="inlineStr">
-        <is>
-          <t>Annual</t>
-        </is>
-      </c>
-      <c r="H31" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I31" s="5" t="inlineStr">
-        <is>
-          <t>Line 27a - Other Expenses</t>
-        </is>
-      </c>
-      <c r="J31" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="B31" s="4" t="n"/>
+      <c r="C31" s="5" t="n"/>
+      <c r="D31" s="5" t="n"/>
+      <c r="E31" s="6" t="n"/>
+      <c r="F31" s="5" t="n"/>
+      <c r="G31" s="5" t="n"/>
+      <c r="H31" s="5" t="n"/>
+      <c r="I31" s="5" t="n"/>
+      <c r="J31" s="5" t="n"/>
       <c r="K31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="B32" s="8" t="n">
-        <v>46089</v>
-      </c>
-      <c r="C32" s="9" t="inlineStr">
-        <is>
-          <t>Marketing/Advertising</t>
-        </is>
-      </c>
-      <c r="D32" s="9" t="inlineStr">
-        <is>
-          <t>1x Google Review</t>
-        </is>
-      </c>
-      <c r="E32" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="F32" s="9" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="G32" s="9" t="inlineStr">
-        <is>
-          <t>One-Time</t>
-        </is>
-      </c>
-      <c r="H32" s="9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I32" s="9" t="inlineStr">
-        <is>
-          <t>Line 8 - Advertising</t>
-        </is>
-      </c>
-      <c r="J32" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="B32" s="8" t="n"/>
+      <c r="C32" s="9" t="n"/>
+      <c r="D32" s="9" t="n"/>
+      <c r="E32" s="10" t="n"/>
+      <c r="F32" s="9" t="n"/>
+      <c r="G32" s="9" t="n"/>
+      <c r="H32" s="9" t="n"/>
+      <c r="I32" s="9" t="n"/>
+      <c r="J32" s="9" t="n"/>
       <c r="K32" s="9" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="B33" s="4" t="n">
-        <v>46090</v>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>Phone/Communications</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>Twilio</t>
-        </is>
-      </c>
-      <c r="E33" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>Credit Card</t>
-        </is>
-      </c>
-      <c r="G33" s="5" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="H33" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I33" s="5" t="inlineStr">
-        <is>
-          <t>Line 25 - Utilities</t>
-        </is>
-      </c>
-      <c r="J33" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="B33" s="4" t="n"/>
+      <c r="C33" s="5" t="n"/>
+      <c r="D33" s="5" t="n"/>
+      <c r="E33" s="6" t="n"/>
+      <c r="F33" s="5" t="n"/>
+      <c r="G33" s="5" t="n"/>
+      <c r="H33" s="5" t="n"/>
+      <c r="I33" s="5" t="n"/>
+      <c r="J33" s="5" t="n"/>
       <c r="K33" s="5" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n">
         <v>32</v>
       </c>
-      <c r="B34" s="8" t="n">
-        <v>46090</v>
-      </c>
-      <c r="C34" s="9" t="inlineStr">
-        <is>
-          <t>Phone/Communications</t>
-        </is>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
-        <is>
-          <t>Quo</t>
-        </is>
-      </c>
-      <c r="E34" s="10" t="n">
-        <v>22.01</v>
-      </c>
-      <c r="F34" s="9" t="inlineStr">
-        <is>
-          <t>ACH/Bank</t>
-        </is>
-      </c>
-      <c r="G34" s="9" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="H34" s="9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I34" s="9" t="inlineStr">
-        <is>
-          <t>Line 25 - Utilities</t>
-        </is>
-      </c>
-      <c r="J34" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="B34" s="8" t="n"/>
+      <c r="C34" s="9" t="n"/>
+      <c r="D34" s="9" t="n"/>
+      <c r="E34" s="10" t="n"/>
+      <c r="F34" s="9" t="n"/>
+      <c r="G34" s="9" t="n"/>
+      <c r="H34" s="9" t="n"/>
+      <c r="I34" s="9" t="n"/>
+      <c r="J34" s="9" t="n"/>
       <c r="K34" s="9" t="n"/>
     </row>
     <row r="35">
@@ -9376,7 +9184,7 @@
       <c r="D3" s="13" t="n"/>
       <c r="E3" s="14" t="n"/>
       <c r="F3" s="6" t="n">
-        <v>35</v>
+        <v>22.68</v>
       </c>
       <c r="G3" s="15" t="n"/>
       <c r="H3" s="5" t="n"/>

</xml_diff>